<commit_message>
Updated Bank Payment And Cash Payment Method
Updated Bank Payment And Cash Payment Method
</commit_message>
<xml_diff>
--- a/testdata/DirectGrnDetailsHK.xlsx
+++ b/testdata/DirectGrnDetailsHK.xlsx
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5914" uniqueCount="251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6230" uniqueCount="399">
   <si>
     <t>Scenario  : Local Purchase - Stock UOM and Purchase UOM (Similar)</t>
   </si>
@@ -816,6 +816,450 @@
   </si>
   <si>
     <t>273.47</t>
+  </si>
+  <si>
+    <t>4956</t>
+  </si>
+  <si>
+    <t>1259.93887</t>
+  </si>
+  <si>
+    <t>4958</t>
+  </si>
+  <si>
+    <t>1259.54451</t>
+  </si>
+  <si>
+    <t>4960</t>
+  </si>
+  <si>
+    <t>1259.15047</t>
+  </si>
+  <si>
+    <t>4962</t>
+  </si>
+  <si>
+    <t>1258.75675</t>
+  </si>
+  <si>
+    <t>5204</t>
+  </si>
+  <si>
+    <t>1245.78715</t>
+  </si>
+  <si>
+    <t>5206</t>
+  </si>
+  <si>
+    <t>1245.41702</t>
+  </si>
+  <si>
+    <t>5208</t>
+  </si>
+  <si>
+    <t>1245.04717</t>
+  </si>
+  <si>
+    <t>5210</t>
+  </si>
+  <si>
+    <t>1244.6776</t>
+  </si>
+  <si>
+    <t>5212</t>
+  </si>
+  <si>
+    <t>1244.30832</t>
+  </si>
+  <si>
+    <t>5214</t>
+  </si>
+  <si>
+    <t>1243.93932</t>
+  </si>
+  <si>
+    <t>5216</t>
+  </si>
+  <si>
+    <t>1243.5706</t>
+  </si>
+  <si>
+    <t>5218</t>
+  </si>
+  <si>
+    <t>1243.20217</t>
+  </si>
+  <si>
+    <t>5220</t>
+  </si>
+  <si>
+    <t>1242.83402</t>
+  </si>
+  <si>
+    <t>5222</t>
+  </si>
+  <si>
+    <t>1242.46615</t>
+  </si>
+  <si>
+    <t>5224</t>
+  </si>
+  <si>
+    <t>1242.09856</t>
+  </si>
+  <si>
+    <t>5226</t>
+  </si>
+  <si>
+    <t>1241.73125</t>
+  </si>
+  <si>
+    <t>5228</t>
+  </si>
+  <si>
+    <t>1241.36423</t>
+  </si>
+  <si>
+    <t>5230</t>
+  </si>
+  <si>
+    <t>1240.99749</t>
+  </si>
+  <si>
+    <t>5268</t>
+  </si>
+  <si>
+    <t>1234.88608</t>
+  </si>
+  <si>
+    <t>5274</t>
+  </si>
+  <si>
+    <t>1233.8024</t>
+  </si>
+  <si>
+    <t>5278</t>
+  </si>
+  <si>
+    <t>1233.08131</t>
+  </si>
+  <si>
+    <t>5282</t>
+  </si>
+  <si>
+    <t>1232.36132</t>
+  </si>
+  <si>
+    <t>5284</t>
+  </si>
+  <si>
+    <t>1232.00173</t>
+  </si>
+  <si>
+    <t>5292</t>
+  </si>
+  <si>
+    <t>1230.5661</t>
+  </si>
+  <si>
+    <t>5296</t>
+  </si>
+  <si>
+    <t>1229.84991</t>
+  </si>
+  <si>
+    <t>5298</t>
+  </si>
+  <si>
+    <t>1229.49222</t>
+  </si>
+  <si>
+    <t>5300</t>
+  </si>
+  <si>
+    <t>1229.1348</t>
+  </si>
+  <si>
+    <t>5304</t>
+  </si>
+  <si>
+    <t>1229.21912</t>
+  </si>
+  <si>
+    <t>5308</t>
+  </si>
+  <si>
+    <t>1229.30331</t>
+  </si>
+  <si>
+    <t>5312</t>
+  </si>
+  <si>
+    <t>1229.38737</t>
+  </si>
+  <si>
+    <t>5316</t>
+  </si>
+  <si>
+    <t>1229.47131</t>
+  </si>
+  <si>
+    <t>5322</t>
+  </si>
+  <si>
+    <t>1229.9948</t>
+  </si>
+  <si>
+    <t>5326</t>
+  </si>
+  <si>
+    <t>1230.07812</t>
+  </si>
+  <si>
+    <t>5330</t>
+  </si>
+  <si>
+    <t>1230.16132</t>
+  </si>
+  <si>
+    <t>5334</t>
+  </si>
+  <si>
+    <t>1230.24439</t>
+  </si>
+  <si>
+    <t>5340</t>
+  </si>
+  <si>
+    <t>1230.76525</t>
+  </si>
+  <si>
+    <t>5344</t>
+  </si>
+  <si>
+    <t>1230.84771</t>
+  </si>
+  <si>
+    <t>5348</t>
+  </si>
+  <si>
+    <t>1230.93005</t>
+  </si>
+  <si>
+    <t>5352</t>
+  </si>
+  <si>
+    <t>1231.01227</t>
+  </si>
+  <si>
+    <t>5360</t>
+  </si>
+  <si>
+    <t>1231.96635</t>
+  </si>
+  <si>
+    <t>5362</t>
+  </si>
+  <si>
+    <t>1231.61214</t>
+  </si>
+  <si>
+    <t>5366</t>
+  </si>
+  <si>
+    <t>1231.69363</t>
+  </si>
+  <si>
+    <t>5370</t>
+  </si>
+  <si>
+    <t>1231.77501</t>
+  </si>
+  <si>
+    <t>5376</t>
+  </si>
+  <si>
+    <t>1232.29067</t>
+  </si>
+  <si>
+    <t>5380</t>
+  </si>
+  <si>
+    <t>1232.37145</t>
+  </si>
+  <si>
+    <t>5386</t>
+  </si>
+  <si>
+    <t>1232.88549</t>
+  </si>
+  <si>
+    <t>6742</t>
+  </si>
+  <si>
+    <t>1154.44195</t>
+  </si>
+  <si>
+    <t>6744</t>
+  </si>
+  <si>
+    <t>1154.18332</t>
+  </si>
+  <si>
+    <t>6746</t>
+  </si>
+  <si>
+    <t>1153.92484</t>
+  </si>
+  <si>
+    <t>6748</t>
+  </si>
+  <si>
+    <t>1153.66651</t>
+  </si>
+  <si>
+    <t>6750</t>
+  </si>
+  <si>
+    <t>1153.40834</t>
+  </si>
+  <si>
+    <t>6752</t>
+  </si>
+  <si>
+    <t>1153.15032</t>
+  </si>
+  <si>
+    <t>6754</t>
+  </si>
+  <si>
+    <t>1152.89245</t>
+  </si>
+  <si>
+    <t>6756</t>
+  </si>
+  <si>
+    <t>1152.63473</t>
+  </si>
+  <si>
+    <t>6760</t>
+  </si>
+  <si>
+    <t>1152.11976</t>
+  </si>
+  <si>
+    <t>6764</t>
+  </si>
+  <si>
+    <t>1151.60539</t>
+  </si>
+  <si>
+    <t>204</t>
+  </si>
+  <si>
+    <t>268.98049</t>
+  </si>
+  <si>
+    <t>6766</t>
+  </si>
+  <si>
+    <t>1151.34844</t>
+  </si>
+  <si>
+    <t>206</t>
+  </si>
+  <si>
+    <t>269.1101</t>
+  </si>
+  <si>
+    <t>6768</t>
+  </si>
+  <si>
+    <t>1151.09164</t>
+  </si>
+  <si>
+    <t>208</t>
+  </si>
+  <si>
+    <t>269.23721</t>
+  </si>
+  <si>
+    <t>6770</t>
+  </si>
+  <si>
+    <t>1150.83499</t>
+  </si>
+  <si>
+    <t>6772</t>
+  </si>
+  <si>
+    <t>1150.57849</t>
+  </si>
+  <si>
+    <t>210</t>
+  </si>
+  <si>
+    <t>269.3619</t>
+  </si>
+  <si>
+    <t>212</t>
+  </si>
+  <si>
+    <t>269.48424</t>
+  </si>
+  <si>
+    <t>6774</t>
+  </si>
+  <si>
+    <t>1150.32214</t>
+  </si>
+  <si>
+    <t>6776</t>
+  </si>
+  <si>
+    <t>1150.06594</t>
+  </si>
+  <si>
+    <t>214</t>
+  </si>
+  <si>
+    <t>269.60429</t>
+  </si>
+  <si>
+    <t>216</t>
+  </si>
+  <si>
+    <t>269.72212</t>
+  </si>
+  <si>
+    <t>6778</t>
+  </si>
+  <si>
+    <t>1149.8099</t>
+  </si>
+  <si>
+    <t>6780</t>
+  </si>
+  <si>
+    <t>1149.55401</t>
+  </si>
+  <si>
+    <t>218</t>
+  </si>
+  <si>
+    <t>269.83779</t>
+  </si>
+  <si>
+    <t>220</t>
+  </si>
+  <si>
+    <t>269.95136</t>
+  </si>
+  <si>
+    <t>6790</t>
+  </si>
+  <si>
+    <t>1148.22025</t>
   </si>
 </sst>
 </file>
@@ -3567,10 +4011,10 @@
       <c r="AT23" s="112" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" s="99" t="s">
+      <c r="AU23" t="s" s="99">
         <v>108</v>
       </c>
-      <c r="AV23" s="99" t="s">
+      <c r="AV23" t="s" s="99">
         <v>149</v>
       </c>
       <c r="AW23" s="112">
@@ -3609,11 +4053,11 @@
       <c r="BL23" s="112" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" s="99" t="s">
-        <v>235</v>
-      </c>
-      <c r="BN23" s="99" t="s">
-        <v>234</v>
+      <c r="BM23" t="s" s="99">
+        <v>392</v>
+      </c>
+      <c r="BN23" t="s" s="99">
+        <v>391</v>
       </c>
       <c r="BO23" s="112">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -57770,10 +58214,10 @@
       <c r="AT23" s="112" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" s="99" t="s">
+      <c r="AU23" t="s" s="99">
         <v>108</v>
       </c>
-      <c r="AV23" s="99" t="s">
+      <c r="AV23" t="s" s="99">
         <v>149</v>
       </c>
       <c r="AW23" s="112">
@@ -57812,11 +58256,11 @@
       <c r="BL23" s="112" t="s">
         <v>222</v>
       </c>
-      <c r="BM23" s="99" t="s">
-        <v>225</v>
-      </c>
-      <c r="BN23" s="99" t="s">
-        <v>173</v>
+      <c r="BM23" t="s" s="99">
+        <v>396</v>
+      </c>
+      <c r="BN23" t="s" s="99">
+        <v>395</v>
       </c>
       <c r="BO23" s="112">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -61845,11 +62289,11 @@
       <c r="AT23" s="112" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" s="99" t="s">
+      <c r="AU23" t="s" s="99">
         <v>108</v>
       </c>
-      <c r="AV23" s="99" t="s">
-        <v>231</v>
+      <c r="AV23" t="s" s="99">
+        <v>188</v>
       </c>
       <c r="AW23" s="112">
         <f>AM23</f>
@@ -61887,11 +62331,11 @@
       <c r="BL23" s="112" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" s="99" t="s">
-        <v>233</v>
-      </c>
-      <c r="BN23" s="99" t="s">
-        <v>232</v>
+      <c r="BM23" t="s" s="99">
+        <v>398</v>
+      </c>
+      <c r="BN23" t="s" s="99">
+        <v>397</v>
       </c>
       <c r="BO23" s="112">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>

</xml_diff>

<commit_message>
ADDED 2 NEW EXCEL FOR THE DIRECT GRN
ADDED 2 NEW EXCEL FOR THE DIRECT GRN
</commit_message>
<xml_diff>
--- a/testdata/DirectGrnDetailsHK.xlsx
+++ b/testdata/DirectGrnDetailsHK.xlsx
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6230" uniqueCount="399">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6286" uniqueCount="417">
   <si>
     <t>Scenario  : Local Purchase - Stock UOM and Purchase UOM (Similar)</t>
   </si>
@@ -1261,6 +1261,60 @@
   <si>
     <t>1148.22025</t>
   </si>
+  <si>
+    <t>6794</t>
+  </si>
+  <si>
+    <t>1148.33372</t>
+  </si>
+  <si>
+    <t>6796</t>
+  </si>
+  <si>
+    <t>1148.70194</t>
+  </si>
+  <si>
+    <t>6798</t>
+  </si>
+  <si>
+    <t>1148.44705</t>
+  </si>
+  <si>
+    <t>6800</t>
+  </si>
+  <si>
+    <t>1148.19231</t>
+  </si>
+  <si>
+    <t>6802</t>
+  </si>
+  <si>
+    <t>1147.93772</t>
+  </si>
+  <si>
+    <t>6804</t>
+  </si>
+  <si>
+    <t>1147.68328</t>
+  </si>
+  <si>
+    <t>6806</t>
+  </si>
+  <si>
+    <t>1147.42899</t>
+  </si>
+  <si>
+    <t>6808</t>
+  </si>
+  <si>
+    <t>1147.17485</t>
+  </si>
+  <si>
+    <t>6810</t>
+  </si>
+  <si>
+    <t>1147.54265</t>
+  </si>
 </sst>
 </file>
 
@@ -4054,10 +4108,10 @@
         <v>148</v>
       </c>
       <c r="BM23" t="s" s="99">
-        <v>392</v>
+        <v>412</v>
       </c>
       <c r="BN23" t="s" s="99">
-        <v>391</v>
+        <v>411</v>
       </c>
       <c r="BO23" s="112">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -62293,7 +62347,7 @@
         <v>108</v>
       </c>
       <c r="AV23" t="s" s="99">
-        <v>188</v>
+        <v>231</v>
       </c>
       <c r="AW23" s="112">
         <f>AM23</f>
@@ -62332,10 +62386,10 @@
         <v>148</v>
       </c>
       <c r="BM23" t="s" s="99">
-        <v>398</v>
+        <v>416</v>
       </c>
       <c r="BN23" t="s" s="99">
-        <v>397</v>
+        <v>415</v>
       </c>
       <c r="BO23" s="112">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>

</xml_diff>